<commit_message>
Source RT/m2 weighted by CBS category, build installed chiller capacity calc
Added Section 3 (RT/m2 sourced per category, flagging the two proxy
categories where no category-specific source exists) and Section 4
(installed chiller capacity by category and year, weighted, live
formulas off Sections 1 and 3) to chiller-market-sizing.xlsx. 5-year
average lands at ~128,600 RT/year from new non-res construction.
Verified independently in Python before shipping since LibreOffice
can't recalc in this sandbox. Also fixed the workbook's own text to
follow the new no-double-hyphen-in-Excel rule.
</commit_message>
<xml_diff>
--- a/projects/energy-program/chiller-market-sizing.xlsx
+++ b/projects/energy-program/chiller-market-sizing.xlsx
@@ -16,8 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="14">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,6 +86,21 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00404040"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
@@ -91,7 +109,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +134,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,8 +209,38 @@
     <xf numFmtId="3" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,19 +608,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
@@ -578,14 +631,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chiller Market Sizing -- CBS Construction-Starts Data (2021-2025)</t>
+          <t>Chiller Market Sizing: CBS Construction-Starts Data (2021-2025)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: Israel Central Bureau of Statistics (הלשכה המרכזית לסטטיסטיקה), "התחלות וגמר בנייה - סיכום שנת 2025" (Construction Begun and Completed in 2025), Publication 089/2026, released 19/03/2026. Table 7 -- Construction area, by purpose and construction stage (CONSTRUCTION BEGUN section).</t>
+          <t>Source: Israel Central Bureau of Statistics (הלשכה המרכזית לסטטיסטיקה), "התחלות וגמר בנייה - סיכום שנת 2025" (Construction Begun and Completed in 2025), Publication 089/2026, released 19/03/2026. Table 7: Construction area, by purpose and construction stage (CONSTRUCTION BEGUN section).</t>
         </is>
       </c>
     </row>
@@ -624,7 +677,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>SECTION 1 -- Raw CBS Data: Construction Begun, by Purpose (Thousand m²)</t>
+          <t>SECTION 1 - Raw CBS Data: Construction Begun, by Purpose (Thousand m²)</t>
         </is>
       </c>
     </row>
@@ -974,21 +1027,21 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>CBS footnote (source table, note 2): "הנתונים אינם מסתכמים בהכרח לסך הכל בגלל עיגול מספרים" -- figures may not sum exactly due to CBS's own rounding. All units: thousand m².</t>
+          <t>CBS footnote (source table, note 2): "הנתונים אינם מסתכמים בהכרח לסך הכל בגלל עיגול מספרים": figures may not sum exactly due to CBS's own rounding. All units: thousand m².</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>SECTION 2 -- Chiller-Relevant Construction Starts (Derived)</t>
+          <t>SECTION 2: Chiller-Relevant Construction Starts (Derived)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Methodology (brainstorms/2026-07-22_tax-incentive-market-analysis.md): chiller-relevant floor area = non-residential total MINUS Agriculture MINUS Transport &amp; communications. These two categories are excluded because they don't carry comfort-cooling loads the way office/commercial/institutional/industrial floor area does. All cells below are live formulas referencing Section 1 -- change a raw CBS input above and this section recalculates.</t>
+          <t>Methodology (brainstorms/2026-07-22_tax-incentive-market-analysis.md): chiller-relevant floor area = non-residential total MINUS Agriculture MINUS Transport &amp; communications. These two categories are excluded because they don't carry comfort-cooling loads the way office/commercial/institutional/industrial floor area does. All cells below are live formulas referencing Section 1: change a raw CBS input above and this section recalculates.</t>
         </is>
       </c>
     </row>
@@ -1180,62 +1233,762 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SECTION 3 -- Notes &amp; Open Questions</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
+          <t>SECTION 3: Cooling-Load Density (RT/m²) by CBS Category, Sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="55" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>No single source publishes one blended commercial-building RT/m² figure, and cooling-load density varies genuinely by building type: so each of the 7 chiller-relevant CBS categories gets its own sourced sq ft/ton figure below, converted to m²/RT via the exact sq-ft-to-m² factor in cell B30. Green rows are directly sourced to a named reference matching that CBS category; orange rows are a general-commercial proxy because no source specific to that category was found: flagged, not hidden. SI 5282 (Israeli standard) was checked and ruled out: it is a building energy-rating standard (envelope, glazing, orientation), not an equipment-capacity sizing standard, so it has no RT/m² figure to cite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Conversion factor: 1 sq ft =</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>0.092903</v>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>m² (exact)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Section 1
+column</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>sq ft / ton
+(sourced input)</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>m² / RT
+(=sqft/ton x conv.)</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
+      <c r="M31" s="8" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Other public buildings</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col C</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="D32" s="22">
+        <f>C32*$B$29</f>
+        <v/>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>Trane (via HVAC industry search compilation): "general commercial" catch-all figure. trane.com/residential/en/resources/glossary/hvac-sizing</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="25" t="inlineStr">
+        <is>
+          <t>Proxy: no source specific to civic/municipal buildings found</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="n"/>
+      <c r="L32" s="24" t="n"/>
+      <c r="M32" s="24" t="n"/>
+      <c r="N32" s="24" t="n"/>
+      <c r="O32" s="24" t="n"/>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Health (בריאות)</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col D</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>275</v>
+      </c>
+      <c r="D33" s="22">
+        <f>C33*$B$29</f>
+        <v/>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>HVAC-ENG.com, Cooling Load Rules of Thumb: patient rooms &amp; medical offices, 250-300 sq ft/ton range, midpoint used. hvac-eng.com/cooling-load-rules-of-thumb</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n"/>
+      <c r="J33" s="28" t="inlineStr">
+        <is>
+          <t>Sourced: matches category directly</t>
+        </is>
+      </c>
+      <c r="K33" s="27" t="n"/>
+      <c r="L33" s="27" t="n"/>
+      <c r="M33" s="27" t="n"/>
+      <c r="N33" s="27" t="n"/>
+      <c r="O33" s="27" t="n"/>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Education (חינוך)</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col E</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="n">
+        <v>213</v>
+      </c>
+      <c r="D34" s="22">
+        <f>C34*$B$29</f>
+        <v/>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>cfm Distributors (Brad Telker, VP Sales), Load Calculation Rules of Thumb: classrooms, stated design assumptions (98/78 db/wb summer design, 2018 IMC ventilation). rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
+      <c r="G34" s="27" t="n"/>
+      <c r="H34" s="27" t="n"/>
+      <c r="I34" s="27" t="n"/>
+      <c r="J34" s="28" t="inlineStr">
+        <is>
+          <t>Sourced: matches category directly</t>
+        </is>
+      </c>
+      <c r="K34" s="27" t="n"/>
+      <c r="L34" s="27" t="n"/>
+      <c r="M34" s="27" t="n"/>
+      <c r="N34" s="27" t="n"/>
+      <c r="O34" s="27" t="n"/>
+    </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Industry &amp; storage</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col F</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="D35" s="22">
+        <f>C35*$B$29</f>
+        <v/>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>Trane (via HVAC industry search compilation): "general commercial" catch-all figure, same as Other public buildings. trane.com/residential/en/resources/glossary/hvac-sizing</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
+      <c r="J35" s="25" t="inlineStr">
+        <is>
+          <t>Proxy: CBS bundles active industrial process floor with pure storage; no disaggregated source found, and HVAC-ENG's industrial figures (50-300 sq ft/ton) are computer-room/precision-manufacturing specific, not general storage</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="n"/>
+      <c r="L35" s="24" t="n"/>
+      <c r="M35" s="24" t="n"/>
+      <c r="N35" s="24" t="n"/>
+      <c r="O35" s="24" t="n"/>
+    </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Commercial (מסחר)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col H</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="n">
+        <v>321</v>
+      </c>
+      <c r="D36" s="22">
+        <f>C36*$B$29</f>
+        <v/>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>cfm Distributors (Brad Telker, VP Sales), Load Calculation Rules of Thumb: retail sales floor. rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+      <c r="H36" s="27" t="n"/>
+      <c r="I36" s="27" t="n"/>
+      <c r="J36" s="28" t="inlineStr">
+        <is>
+          <t>Sourced: matches category directly</t>
+        </is>
+      </c>
+      <c r="K36" s="27" t="n"/>
+      <c r="L36" s="27" t="n"/>
+      <c r="M36" s="27" t="n"/>
+      <c r="N36" s="27" t="n"/>
+      <c r="O36" s="27" t="n"/>
+    </row>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Offices (משרדים)</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col I</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="n">
+        <v>373</v>
+      </c>
+      <c r="D37" s="22">
+        <f>C37*$B$29</f>
+        <v/>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>cfm Distributors (Brad Telker, VP Sales), Load Calculation Rules of Thumb: office space. rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
+      <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n"/>
+      <c r="J37" s="28" t="inlineStr">
+        <is>
+          <t>Sourced: matches category directly</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="n"/>
+      <c r="L37" s="27" t="n"/>
+      <c r="M37" s="27" t="n"/>
+      <c r="N37" s="27" t="n"/>
+      <c r="O37" s="27" t="n"/>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Hotels (הארחה)</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="inlineStr">
+        <is>
+          <t>Section 1, col J</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="n">
+        <v>362.5</v>
+      </c>
+      <c r="D38" s="22">
+        <f>C38*$B$29</f>
+        <v/>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>HVAC-ENG.com, Cooling Load Rules of Thumb: unweighted average of public spaces (250-300, mid 275) and guest rooms (400-500, mid 450); no hotel floor-area split between the two is sourced. hvac-eng.com/cooling-load-rules-of-thumb</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n"/>
+      <c r="G38" s="27" t="n"/>
+      <c r="H38" s="27" t="n"/>
+      <c r="I38" s="27" t="n"/>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>Sourced but blended: no public/guest-room area split available</t>
+        </is>
+      </c>
+      <c r="K38" s="27" t="n"/>
+      <c r="L38" s="27" t="n"/>
+      <c r="M38" s="27" t="n"/>
+      <c r="N38" s="27" t="n"/>
+      <c r="O38" s="27" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>SECTION 4: Installed Chiller Capacity by Category and Year (Weighted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Per-category RT = (Section 1 m², thousand) x 1000 / (Section 3 m²/RT for that category). Summed across the 7 chiller-relevant categories = total new chiller capacity (RT) added that year. "Blended m²/RT (check)" divides total chiller-relevant m² by total RT: a reference figure showing what single blended ratio this year's actual construction mix implies, for comparison against a flat assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Other public
+(RT)</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Health
+(RT)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Education
+(RT)</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Industry &amp; storage
+(RT)</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Commercial
+(RT)</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Offices
+(RT)</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Hotels
+(RT)</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>Total
+(RT)</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Blended m²/RT
+(check)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13">
+        <f>A8</f>
+        <v/>
+      </c>
+      <c r="B44" s="11">
+        <f>C8*1000/$D$32</f>
+        <v/>
+      </c>
+      <c r="C44" s="11">
+        <f>D8*1000/$D$33</f>
+        <v/>
+      </c>
+      <c r="D44" s="11">
+        <f>E8*1000/$D$34</f>
+        <v/>
+      </c>
+      <c r="E44" s="11">
+        <f>F8*1000/$D$35</f>
+        <v/>
+      </c>
+      <c r="F44" s="11">
+        <f>H8*1000/$D$36</f>
+        <v/>
+      </c>
+      <c r="G44" s="11">
+        <f>I8*1000/$D$37</f>
+        <v/>
+      </c>
+      <c r="H44" s="11">
+        <f>J8*1000/$D$38</f>
+        <v/>
+      </c>
+      <c r="I44" s="14">
+        <f>SUM(B44:H44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="29">
+        <f>F20/I44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13">
+        <f>A9</f>
+        <v/>
+      </c>
+      <c r="B45" s="11">
+        <f>C9*1000/$D$32</f>
+        <v/>
+      </c>
+      <c r="C45" s="11">
+        <f>D9*1000/$D$33</f>
+        <v/>
+      </c>
+      <c r="D45" s="11">
+        <f>E9*1000/$D$34</f>
+        <v/>
+      </c>
+      <c r="E45" s="11">
+        <f>F9*1000/$D$35</f>
+        <v/>
+      </c>
+      <c r="F45" s="11">
+        <f>H9*1000/$D$36</f>
+        <v/>
+      </c>
+      <c r="G45" s="11">
+        <f>I9*1000/$D$37</f>
+        <v/>
+      </c>
+      <c r="H45" s="11">
+        <f>J9*1000/$D$38</f>
+        <v/>
+      </c>
+      <c r="I45" s="14">
+        <f>SUM(B45:H45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="29">
+        <f>F21/I45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13">
+        <f>A10</f>
+        <v/>
+      </c>
+      <c r="B46" s="11">
+        <f>C10*1000/$D$32</f>
+        <v/>
+      </c>
+      <c r="C46" s="11">
+        <f>D10*1000/$D$33</f>
+        <v/>
+      </c>
+      <c r="D46" s="11">
+        <f>E10*1000/$D$34</f>
+        <v/>
+      </c>
+      <c r="E46" s="11">
+        <f>F10*1000/$D$35</f>
+        <v/>
+      </c>
+      <c r="F46" s="11">
+        <f>H10*1000/$D$36</f>
+        <v/>
+      </c>
+      <c r="G46" s="11">
+        <f>I10*1000/$D$37</f>
+        <v/>
+      </c>
+      <c r="H46" s="11">
+        <f>J10*1000/$D$38</f>
+        <v/>
+      </c>
+      <c r="I46" s="14">
+        <f>SUM(B46:H46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="29">
+        <f>F22/I46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13">
+        <f>A11</f>
+        <v/>
+      </c>
+      <c r="B47" s="11">
+        <f>C11*1000/$D$32</f>
+        <v/>
+      </c>
+      <c r="C47" s="11">
+        <f>D11*1000/$D$33</f>
+        <v/>
+      </c>
+      <c r="D47" s="11">
+        <f>E11*1000/$D$34</f>
+        <v/>
+      </c>
+      <c r="E47" s="11">
+        <f>F11*1000/$D$35</f>
+        <v/>
+      </c>
+      <c r="F47" s="11">
+        <f>H11*1000/$D$36</f>
+        <v/>
+      </c>
+      <c r="G47" s="11">
+        <f>I11*1000/$D$37</f>
+        <v/>
+      </c>
+      <c r="H47" s="11">
+        <f>J11*1000/$D$38</f>
+        <v/>
+      </c>
+      <c r="I47" s="14">
+        <f>SUM(B47:H47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="29">
+        <f>F23/I47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13">
+        <f>A12</f>
+        <v/>
+      </c>
+      <c r="B48" s="11">
+        <f>C12*1000/$D$32</f>
+        <v/>
+      </c>
+      <c r="C48" s="11">
+        <f>D12*1000/$D$33</f>
+        <v/>
+      </c>
+      <c r="D48" s="11">
+        <f>E12*1000/$D$34</f>
+        <v/>
+      </c>
+      <c r="E48" s="11">
+        <f>F12*1000/$D$35</f>
+        <v/>
+      </c>
+      <c r="F48" s="11">
+        <f>H12*1000/$D$36</f>
+        <v/>
+      </c>
+      <c r="G48" s="11">
+        <f>I12*1000/$D$37</f>
+        <v/>
+      </c>
+      <c r="H48" s="11">
+        <f>J12*1000/$D$38</f>
+        <v/>
+      </c>
+      <c r="I48" s="14">
+        <f>SUM(B48:H48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="29">
+        <f>F24/I48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>5-yr average</t>
+        </is>
+      </c>
+      <c r="B49" s="17">
+        <f>AVERAGE(B44:B48)</f>
+        <v/>
+      </c>
+      <c r="C49" s="17">
+        <f>AVERAGE(C44:C48)</f>
+        <v/>
+      </c>
+      <c r="D49" s="17">
+        <f>AVERAGE(D44:D48)</f>
+        <v/>
+      </c>
+      <c r="E49" s="17">
+        <f>AVERAGE(E44:E48)</f>
+        <v/>
+      </c>
+      <c r="F49" s="17">
+        <f>AVERAGE(F44:F48)</f>
+        <v/>
+      </c>
+      <c r="G49" s="17">
+        <f>AVERAGE(G44:G48)</f>
+        <v/>
+      </c>
+      <c r="H49" s="17">
+        <f>AVERAGE(H44:H48)</f>
+        <v/>
+      </c>
+      <c r="I49" s="14">
+        <f>AVERAGE(I44:I48)</f>
+        <v/>
+      </c>
+      <c r="J49" s="31">
+        <f>AVERAGE(J44:J48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>SECTION 5: Notes &amp; Open Questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="75" customHeight="1">
+      <c r="A52" s="32" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>5-year average chiller-relevant construction starts ≈ 3,965 thousand m²/year (~3.97M m²/year), cell E/F on the 5-yr average row above. No strong up/down trend -- 2023 was a peak (4,546k), 2024 a trough (3,192k), plausibly tied to construction-sector disruption since the war started (Oct 2023), which CBS's own release separately documents (labor shortages, security-related site disruptions). A flat 5-year average was used as the growth parameter rather than a fitted trend line, since the 2023-2024 swing makes a trend fit noisy rather than more informative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>Open question for Daniel</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>CBS bundles "Industry &amp; storage" as a single category (column F, Section 1). Pure storage/warehousing space often doesn't carry the same comfort/process cooling load as active industrial floor space, but CBS provides no further breakdown at this level of the release. Flagging as a methodology call rather than guessing a split -- would need a different data source to split it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="B52" s="33" t="inlineStr">
+        <is>
+          <t>5-year average weighted installed chiller capacity from new non-residential construction ≈ 128,600 RT/year (cell I49). The blended m²/RT this implies each year (column J, Section 4) stays fairly stable at ~30-31.5 m²/RT despite year-to-year swings in category mix, because Education (dense, ~19.8 m²/RT) and the two proxy categories (less dense, ~37.2 m²/RT) partly offset each other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="75" customHeight="1">
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>Open question for Daniel: proxy categories</t>
+        </is>
+      </c>
+      <c r="B53" s="33" t="inlineStr">
+        <is>
+          <t>"Other public buildings" and "Industry &amp; storage" (Section 3, orange rows) both use a general-commercial proxy figure (Trane, 400 sq ft/ton) because no source specific to either category was found. This is the weakest link in the weighted calc: industrial/storage floor space in particular could plausibly be much lower cooling-load than a flat commercial proxy assumes (empty warehouse space often isn't fully air-conditioned at all). Flagging rather than guessing a differentiated number with no basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="75" customHeight="1">
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>Open question for Daniel: CBS bundling</t>
+        </is>
+      </c>
+      <c r="B54" s="33" t="inlineStr">
+        <is>
+          <t>CBS bundles "Industry &amp; storage" as a single category (Section 1, column F) with no further breakdown at this release level: pure storage/warehousing likely doesn't carry the same load as active industrial floor space, but there's no CBS-level way to split it. Would need a different data source (e.g. PRTR facility-level data, already flagged as a lead for the HP/VSD sizing engines) to separate them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="75" customHeight="1">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t>Not yet built</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>RT/m² (cooling-load density) still needs sourcing (ASHRAE rule-of-thumb or Israeli standard SI 5282) to convert the chiller-relevant m²/year figure above into installed cooling capacity (RT/year) -- that's the next step in the sizing engine, not yet in this workbook.</t>
+      <c r="B55" s="33" t="inlineStr">
+        <is>
+          <t>Replacement-demand sensitivity (existing stock RT / equipment lifetime, per the model's own 15-17yr lifetime rows) is still the next step: this workbook covers new-construction demand only, the conservative base case per the market-sizing methodology doc.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="35">
+    <mergeCell ref="A16:O16"/>
+    <mergeCell ref="A41:O41"/>
+    <mergeCell ref="B54:O54"/>
+    <mergeCell ref="J36:O36"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="A27:O27"/>
+    <mergeCell ref="J35:O35"/>
+    <mergeCell ref="E35:I35"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="J32:O32"/>
+    <mergeCell ref="B52:O52"/>
+    <mergeCell ref="A14:O14"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="J31:O31"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="A17:O17"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="B53:O53"/>
+    <mergeCell ref="J33:O33"/>
+    <mergeCell ref="A28:O28"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="A40:O40"/>
+    <mergeCell ref="J38:O38"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="A16:O16"/>
-    <mergeCell ref="L3:O3"/>
-    <mergeCell ref="B30:O30"/>
-    <mergeCell ref="A14:O14"/>
-    <mergeCell ref="B29:O29"/>
+    <mergeCell ref="A51:O51"/>
+    <mergeCell ref="J37:O37"/>
+    <mergeCell ref="B55:O55"/>
+    <mergeCell ref="E32:I32"/>
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A27:O27"/>
-    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="E37:I37"/>
     <mergeCell ref="A6:O6"/>
-    <mergeCell ref="B28:O28"/>
-    <mergeCell ref="A17:O17"/>
+    <mergeCell ref="J34:O34"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>

</xml_diff>

<commit_message>
Capture the industry/storage proxy tension for the Daniel/Rafi conversation
Omri flagged that the 400 sqft/ton proxy makes Industry & storage read
as the least cooling-intensive category, which cuts against intuition
about industrial process cooling. Documented both sides of the tension
(CBS bundling active industrial floor with pure storage vs. Daniel's
"comfort chillers" comment on the core model's hours assumption) in
the workbook's notes and market-analysis.md, flagged as unresolved
pending a direct conversation with Daniel/Rafi on chiller scope.
</commit_message>
<xml_diff>
--- a/projects/energy-program/chiller-market-sizing.xlsx
+++ b/projects/energy-program/chiller-market-sizing.xlsx
@@ -205,7 +205,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -243,11 +243,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -364,6 +408,8 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1421,20 +1467,20 @@
           <t>מקור</t>
         </is>
       </c>
-      <c r="F31" s="31" t="n"/>
-      <c r="G31" s="31" t="n"/>
-      <c r="H31" s="31" t="n"/>
-      <c r="I31" s="31" t="n"/>
+      <c r="F31" s="52" t="n"/>
+      <c r="G31" s="52" t="n"/>
+      <c r="H31" s="52" t="n"/>
+      <c r="I31" s="53" t="n"/>
       <c r="J31" s="31" t="inlineStr">
         <is>
           <t>בסיס</t>
         </is>
       </c>
-      <c r="K31" s="31" t="n"/>
-      <c r="L31" s="31" t="n"/>
-      <c r="M31" s="31" t="n"/>
-      <c r="N31" s="31" t="n"/>
-      <c r="O31" s="31" t="n"/>
+      <c r="K31" s="52" t="n"/>
+      <c r="L31" s="52" t="n"/>
+      <c r="M31" s="52" t="n"/>
+      <c r="N31" s="52" t="n"/>
+      <c r="O31" s="53" t="n"/>
     </row>
     <row r="32" ht="60" customHeight="1" s="22">
       <c r="A32" s="32" t="inlineStr">
@@ -1459,20 +1505,20 @@
           <t>Trane (מתוך ליקוט מקורות תעשיית ה-HVAC) - מקדם כללי ל"מסחרי כללי". trane.com/residential/en/resources/glossary/hvac-sizing</t>
         </is>
       </c>
-      <c r="F32" s="37" t="n"/>
-      <c r="G32" s="37" t="n"/>
-      <c r="H32" s="37" t="n"/>
-      <c r="I32" s="37" t="n"/>
+      <c r="F32" s="52" t="n"/>
+      <c r="G32" s="52" t="n"/>
+      <c r="H32" s="52" t="n"/>
+      <c r="I32" s="53" t="n"/>
       <c r="J32" s="38" t="inlineStr">
         <is>
           <t>פרוקסי - לא נמצא מקור ספציפי למבני ציבור/עירייה</t>
         </is>
       </c>
-      <c r="K32" s="37" t="n"/>
-      <c r="L32" s="37" t="n"/>
-      <c r="M32" s="37" t="n"/>
-      <c r="N32" s="37" t="n"/>
-      <c r="O32" s="37" t="n"/>
+      <c r="K32" s="52" t="n"/>
+      <c r="L32" s="52" t="n"/>
+      <c r="M32" s="52" t="n"/>
+      <c r="N32" s="52" t="n"/>
+      <c r="O32" s="53" t="n"/>
     </row>
     <row r="33" ht="60" customHeight="1" s="22">
       <c r="A33" s="32" t="inlineStr">
@@ -1497,20 +1543,20 @@
           <t>HVAC-ENG.com, Cooling Load Rules of Thumb - חדרי מטופלים ומרפאות, טווח 250-300 רגל רבועה/טון, נעשה שימוש בנקודת האמצע. hvac-eng.com/cooling-load-rules-of-thumb</t>
         </is>
       </c>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="40" t="n"/>
-      <c r="H33" s="40" t="n"/>
-      <c r="I33" s="40" t="n"/>
+      <c r="F33" s="52" t="n"/>
+      <c r="G33" s="52" t="n"/>
+      <c r="H33" s="52" t="n"/>
+      <c r="I33" s="53" t="n"/>
       <c r="J33" s="41" t="inlineStr">
         <is>
           <t>מקור ישיר - תואם את הקטגוריה במדויק</t>
         </is>
       </c>
-      <c r="K33" s="40" t="n"/>
-      <c r="L33" s="40" t="n"/>
-      <c r="M33" s="40" t="n"/>
-      <c r="N33" s="40" t="n"/>
-      <c r="O33" s="40" t="n"/>
+      <c r="K33" s="52" t="n"/>
+      <c r="L33" s="52" t="n"/>
+      <c r="M33" s="52" t="n"/>
+      <c r="N33" s="52" t="n"/>
+      <c r="O33" s="53" t="n"/>
     </row>
     <row r="34" ht="60" customHeight="1" s="22">
       <c r="A34" s="32" t="inlineStr">
@@ -1535,20 +1581,20 @@
           <t>cfm Distributors (Brad Telker, סמנכ"ל מכירות), Load Calculation Rules of Thumb - כיתות לימוד, הנחות תכנון מוצהרות (עיצוב קיץ 98/78 יבש/רטוב, אוורור לפי 2018 IMC). rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
         </is>
       </c>
-      <c r="F34" s="40" t="n"/>
-      <c r="G34" s="40" t="n"/>
-      <c r="H34" s="40" t="n"/>
-      <c r="I34" s="40" t="n"/>
+      <c r="F34" s="52" t="n"/>
+      <c r="G34" s="52" t="n"/>
+      <c r="H34" s="52" t="n"/>
+      <c r="I34" s="53" t="n"/>
       <c r="J34" s="41" t="inlineStr">
         <is>
           <t>מקור ישיר - תואם את הקטגוריה במדויק</t>
         </is>
       </c>
-      <c r="K34" s="40" t="n"/>
-      <c r="L34" s="40" t="n"/>
-      <c r="M34" s="40" t="n"/>
-      <c r="N34" s="40" t="n"/>
-      <c r="O34" s="40" t="n"/>
+      <c r="K34" s="52" t="n"/>
+      <c r="L34" s="52" t="n"/>
+      <c r="M34" s="52" t="n"/>
+      <c r="N34" s="52" t="n"/>
+      <c r="O34" s="53" t="n"/>
     </row>
     <row r="35" ht="60" customHeight="1" s="22">
       <c r="A35" s="32" t="inlineStr">
@@ -1573,20 +1619,20 @@
           <t>Trane (מתוך ליקוט מקורות תעשיית ה-HVAC) - מקדם כללי ל"מסחרי כללי", זהה למבני ציבור אחרים. trane.com/residential/en/resources/glossary/hvac-sizing</t>
         </is>
       </c>
-      <c r="F35" s="37" t="n"/>
-      <c r="G35" s="37" t="n"/>
-      <c r="H35" s="37" t="n"/>
-      <c r="I35" s="37" t="n"/>
+      <c r="F35" s="52" t="n"/>
+      <c r="G35" s="52" t="n"/>
+      <c r="H35" s="52" t="n"/>
+      <c r="I35" s="53" t="n"/>
       <c r="J35" s="38" t="inlineStr">
         <is>
           <t>פרוקסי - הלמ"ס מאחדת שטח תעשייתי פעיל עם אחסון טהור; לא נמצא מקור מפורק</t>
         </is>
       </c>
-      <c r="K35" s="37" t="n"/>
-      <c r="L35" s="37" t="n"/>
-      <c r="M35" s="37" t="n"/>
-      <c r="N35" s="37" t="n"/>
-      <c r="O35" s="37" t="n"/>
+      <c r="K35" s="52" t="n"/>
+      <c r="L35" s="52" t="n"/>
+      <c r="M35" s="52" t="n"/>
+      <c r="N35" s="52" t="n"/>
+      <c r="O35" s="53" t="n"/>
     </row>
     <row r="36" ht="60" customHeight="1" s="22">
       <c r="A36" s="32" t="inlineStr">
@@ -1611,20 +1657,20 @@
           <t>cfm Distributors (Brad Telker, סמנכ"ל מכירות), Load Calculation Rules of Thumb - רצפת מכירות קמעונאית. rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
         </is>
       </c>
-      <c r="F36" s="40" t="n"/>
-      <c r="G36" s="40" t="n"/>
-      <c r="H36" s="40" t="n"/>
-      <c r="I36" s="40" t="n"/>
+      <c r="F36" s="52" t="n"/>
+      <c r="G36" s="52" t="n"/>
+      <c r="H36" s="52" t="n"/>
+      <c r="I36" s="53" t="n"/>
       <c r="J36" s="41" t="inlineStr">
         <is>
           <t>מקור ישיר - תואם את הקטגוריה במדויק</t>
         </is>
       </c>
-      <c r="K36" s="40" t="n"/>
-      <c r="L36" s="40" t="n"/>
-      <c r="M36" s="40" t="n"/>
-      <c r="N36" s="40" t="n"/>
-      <c r="O36" s="40" t="n"/>
+      <c r="K36" s="52" t="n"/>
+      <c r="L36" s="52" t="n"/>
+      <c r="M36" s="52" t="n"/>
+      <c r="N36" s="52" t="n"/>
+      <c r="O36" s="53" t="n"/>
     </row>
     <row r="37" ht="60" customHeight="1" s="22">
       <c r="A37" s="32" t="inlineStr">
@@ -1649,20 +1695,20 @@
           <t>cfm Distributors (Brad Telker, סמנכ"ל מכירות), Load Calculation Rules of Thumb - שטח משרדים. rc.cfmdistributors.com/helpful-tips/training/load-calculation-rules-of-thumb</t>
         </is>
       </c>
-      <c r="F37" s="40" t="n"/>
-      <c r="G37" s="40" t="n"/>
-      <c r="H37" s="40" t="n"/>
-      <c r="I37" s="40" t="n"/>
+      <c r="F37" s="52" t="n"/>
+      <c r="G37" s="52" t="n"/>
+      <c r="H37" s="52" t="n"/>
+      <c r="I37" s="53" t="n"/>
       <c r="J37" s="41" t="inlineStr">
         <is>
           <t>מקור ישיר - תואם את הקטגוריה במדויק</t>
         </is>
       </c>
-      <c r="K37" s="40" t="n"/>
-      <c r="L37" s="40" t="n"/>
-      <c r="M37" s="40" t="n"/>
-      <c r="N37" s="40" t="n"/>
-      <c r="O37" s="40" t="n"/>
+      <c r="K37" s="52" t="n"/>
+      <c r="L37" s="52" t="n"/>
+      <c r="M37" s="52" t="n"/>
+      <c r="N37" s="52" t="n"/>
+      <c r="O37" s="53" t="n"/>
     </row>
     <row r="38" ht="60" customHeight="1" s="22">
       <c r="A38" s="32" t="inlineStr">
@@ -1687,20 +1733,20 @@
           <t>HVAC-ENG.com, Cooling Load Rules of Thumb - ממוצע לא משוקלל בין שטחים ציבוריים (250-300, אמצע 275) לחדרי אורחים (400-500, אמצע 450); לא נמצא מקור לחלוקת השטח בין השניים. hvac-eng.com/cooling-load-rules-of-thumb</t>
         </is>
       </c>
-      <c r="F38" s="40" t="n"/>
-      <c r="G38" s="40" t="n"/>
-      <c r="H38" s="40" t="n"/>
-      <c r="I38" s="40" t="n"/>
+      <c r="F38" s="52" t="n"/>
+      <c r="G38" s="52" t="n"/>
+      <c r="H38" s="52" t="n"/>
+      <c r="I38" s="53" t="n"/>
       <c r="J38" s="41" t="inlineStr">
         <is>
           <t>מקור עם מיזוג - אין חלוקת שטח מקורית בין הקטגוריות</t>
         </is>
       </c>
-      <c r="K38" s="40" t="n"/>
-      <c r="L38" s="40" t="n"/>
-      <c r="M38" s="40" t="n"/>
-      <c r="N38" s="40" t="n"/>
-      <c r="O38" s="40" t="n"/>
+      <c r="K38" s="52" t="n"/>
+      <c r="L38" s="52" t="n"/>
+      <c r="M38" s="52" t="n"/>
+      <c r="N38" s="52" t="n"/>
+      <c r="O38" s="53" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="42" t="inlineStr">
@@ -2073,7 +2119,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="75" customHeight="1" s="22">
+    <row r="55" ht="120" customHeight="1" s="22">
       <c r="A55" s="50" t="inlineStr">
         <is>
           <t>שאלה פתוחה - קטגוריות פרוקסי</t>
@@ -2081,7 +2127,7 @@
       </c>
       <c r="B55" s="51" t="inlineStr">
         <is>
-          <t>"מבני ציבור אחרים" ו"תעשייה ואחסנה" (חלק 3, שורות כתומות) משתמשות שתיהן בנתון פרוקסי מסחרי כללי (Trane, 400 רגל רבועה/טון) משום שלא נמצא מקור ספציפי לאף אחת מהקטגוריות. זהו החוליה החלשה ביותר בחישוב המשוקלל - שטח תעשייה/אחסון בפרט עשוי להיות בעל עומס קירור נמוך משמעותית מהנחת ברירת מחדל מסחרית שטוחה (שטח מחסנים ריק לעיתים קרובות אינו ממוזג כלל). מסומן ולא מוסתר, כדי לא לנחש מספר מבודל ללא בסיס.</t>
+          <t>"מבני ציבור אחרים" ו"תעשייה ואחסנה" (חלק 3, שורות כתומות) משתמשות שתיהן בנתון פרוקסי מסחרי כללי (Trane, 400 רגל רבועה/טון) משום שלא נמצא מקור ספציפי לאף אחת מהקטגוריות. זו החוליה החלשה ביותר בחישוב המשוקלל, ועדיין פתוחה לדיון עם דניאל ורפי. שני שיקולים מושכים לכיוונים מנוגדים: מצד אחד, הלמ"ס מאחדת שטח תעשייתי פעיל (שעשוי לדרוש קירור תהליכי אינטנסיבי) עם אחסון טהור (לרוב לא ממוזג כלל - כ-45% מהמחסנים אינם מקוררים לפי מקור אחד שנבדק) - כך שהתמהיל בפועל לא ידוע. מצד שני, דניאל אישר בדיון על הנחת שעות העבודה במודל התמריץ המרכזי ש-3,000 שעות/שנה זו הנחה טובה "במיוחד לצ'ילרים לנוחות" - ניסוח שמרמז שהיקף הצ'ילרים במודל הוא קירור נוחות למבנה ולא קירור תהליכי, מה שדווקא תומך בכיוון של עומס קירור נמוך יותר (לא גבוה יותר) לשטח תעשייה. לא הוכרע - דורש בירור ישיר מול דניאל/רפי לגבי היקף טכנולוגיית הצ'ילרים במודל: קירור נוחות בלבד, או גם קירור תהליכי.</t>
         </is>
       </c>
     </row>

</xml_diff>